<commit_message>
boton cargar recetas desde excel con deteccion variantes
</commit_message>
<xml_diff>
--- a/Mp Catering _ Recetas para sistema Mariana.xlsx
+++ b/Mp Catering _ Recetas para sistema Mariana.xlsx
@@ -5,15 +5,15 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lcoci\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lcoci\OneDrive\Desktop\mpcatering\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEFC857B-9AEF-49C0-8563-43D3FA911317}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B910B69-C91A-4856-A046-79BC7CE6D64F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="20715" windowHeight="13155" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Solapa Ejemplo" sheetId="1" r:id="rId1"/>
+    <sheet name="Hoja 1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>Ingrediente</t>
   </si>
@@ -50,25 +50,10 @@
     <t>Nombre de Plato</t>
   </si>
   <si>
-    <t>Salsa Blanca</t>
-  </si>
-  <si>
-    <t>Roux</t>
-  </si>
-  <si>
     <t>Porciones que salieron</t>
   </si>
   <si>
-    <t>Nuez Moscada</t>
-  </si>
-  <si>
     <t>Peso por porcion (por formula no tocar)</t>
-  </si>
-  <si>
-    <t>Leche</t>
-  </si>
-  <si>
-    <t>Manteca</t>
   </si>
   <si>
     <t>1.</t>
@@ -78,6 +63,15 @@
   </si>
   <si>
     <t>Cargada en sistema</t>
+  </si>
+  <si>
+    <t>SANGUCHE</t>
+  </si>
+  <si>
+    <t>JAMON</t>
+  </si>
+  <si>
+    <t>QUESO</t>
   </si>
 </sst>
 </file>
@@ -439,7 +433,7 @@
         <v>4</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="H1" s="5"/>
       <c r="I1" s="5"/>
@@ -464,20 +458,20 @@
     </row>
     <row r="2" spans="1:27" ht="13.15" x14ac:dyDescent="0.35">
       <c r="A2" s="6" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="B2" s="7">
         <v>1</v>
       </c>
       <c r="C2" s="7">
-        <v>0.4</v>
+        <v>1</v>
       </c>
       <c r="D2" s="8">
         <f t="shared" ref="D2:D256" si="0">IFERROR((B2-C2)/B2,"")</f>
-        <v>0.6</v>
+        <v>0</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="G2" s="4">
         <v>10</v>
@@ -485,24 +479,24 @@
     </row>
     <row r="3" spans="1:27" ht="13.15" x14ac:dyDescent="0.35">
       <c r="A3" s="6" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="B3" s="7">
-        <v>2E-3</v>
+        <v>1</v>
       </c>
       <c r="C3" s="7">
-        <v>2E-3</v>
+        <v>1</v>
       </c>
       <c r="D3" s="8">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="G3" s="9">
         <f>SUM(B2:B1000)/G2</f>
-        <v>0.20019999999999999</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="4" spans="1:27" ht="12.75" x14ac:dyDescent="0.35">
@@ -515,39 +509,21 @@
       </c>
     </row>
     <row r="5" spans="1:27" ht="12.75" x14ac:dyDescent="0.35">
-      <c r="A5" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="B5" s="7">
-        <v>0.5</v>
-      </c>
-      <c r="C5" s="7">
-        <v>0.5</v>
-      </c>
-      <c r="D5" s="8">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
+      <c r="A5" s="6"/>
+      <c r="B5" s="7"/>
+      <c r="C5" s="7"/>
+      <c r="D5" s="8"/>
     </row>
     <row r="6" spans="1:27" ht="12.75" x14ac:dyDescent="0.35">
-      <c r="A6" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="B6" s="7">
-        <v>0.5</v>
-      </c>
-      <c r="C6" s="7">
-        <v>0.5</v>
-      </c>
-      <c r="D6" s="8">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
+      <c r="A6" s="6"/>
+      <c r="B6" s="7"/>
+      <c r="C6" s="7"/>
+      <c r="D6" s="8"/>
       <c r="F6" s="10" t="s">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="G6" s="11" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
     </row>
     <row r="7" spans="1:27" ht="12.75" x14ac:dyDescent="0.35">
@@ -562,7 +538,7 @@
         <v>1</v>
       </c>
       <c r="G7" s="11" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8" spans="1:27" ht="12.75" x14ac:dyDescent="0.35">

</xml_diff>